<commit_message>
sheets upload and responsive classes
</commit_message>
<xml_diff>
--- a/families.xlsx
+++ b/families.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28014"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\marmina\api\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\marmina\api\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B0BC1F-C318-4F89-9236-D15EB4B7CE1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336"/>
   </bookViews>
   <sheets>
     <sheet name="ورقة1" sheetId="1" r:id="rId1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
   <si>
     <t>id</t>
   </si>
@@ -108,9 +107,6 @@
     <t>سنه خامسه كبار</t>
   </si>
   <si>
-    <t>المرحلة الثالثه كبار</t>
-  </si>
-  <si>
     <t>مرحلة خاصة</t>
   </si>
   <si>
@@ -127,12 +123,18 @@
   </si>
   <si>
     <t>stage</t>
+  </si>
+  <si>
+    <t>المرحلة الثالثة ع ث</t>
+  </si>
+  <si>
+    <t>المرحلة الرابعة ع ث</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -443,13 +445,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="23.6640625" customWidth="1"/>
     <col min="3" max="3" width="23.33203125" customWidth="1"/>
-    <col min="4" max="4" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -463,7 +465,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -561,7 +563,7 @@
         <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -575,7 +577,7 @@
         <v>24</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -589,7 +591,7 @@
         <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -603,7 +605,7 @@
         <v>26</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -611,13 +613,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" t="s">
         <v>31</v>
       </c>
-      <c r="C12" t="s">
-        <v>32</v>
-      </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -631,7 +633,7 @@
         <v>10</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -639,13 +641,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
results and next_family fix
</commit_message>
<xml_diff>
--- a/families.xlsx
+++ b/families.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\marmina\api\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0873D8FD-14CF-410E-804F-F2FE228E9B65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ورقة1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="36">
   <si>
     <t>id</t>
   </si>
@@ -129,12 +130,15 @@
   </si>
   <si>
     <t>المرحلة الرابعة ع ث</t>
+  </si>
+  <si>
+    <t>next_family</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -164,8 +168,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -445,16 +452,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D14"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="23.6640625" customWidth="1"/>
     <col min="3" max="3" width="23.33203125" customWidth="1"/>
-    <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" customWidth="1"/>
+    <col min="5" max="5" width="35.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -467,8 +476,11 @@
       <c r="D1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -481,8 +493,11 @@
       <c r="D2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -495,8 +510,11 @@
       <c r="D3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -509,8 +527,11 @@
       <c r="D4" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -523,8 +544,11 @@
       <c r="D5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -537,8 +561,11 @@
       <c r="D6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -551,8 +578,11 @@
       <c r="D7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -565,8 +595,11 @@
       <c r="D8" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -579,8 +612,11 @@
       <c r="D9" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -593,8 +629,11 @@
       <c r="D10" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -607,8 +646,11 @@
       <c r="D11" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -622,7 +664,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -636,7 +678,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>

</xml_diff>